<commit_message>
fix: resolve registration validation failures and align role parameter
</commit_message>
<xml_diff>
--- a/selenium-tests/E2E_Test_Report.xlsx
+++ b/selenium-tests/E2E_Test_Report.xlsx
@@ -701,7 +701,7 @@
     <t>Success registration of new standard user</t>
   </si>
   <si>
-    <t>Name: "New Test Patient", Phone: "9876543210", Email: "reg_valid_1782125671329@example.com"</t>
+    <t>Name: "New Test Patient", Phone: "9876543210", Email: "reg_valid_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Success redirect to user dashboard</t>
@@ -725,7 +725,7 @@
     <t>Registration failure with short password (&lt;6 chars)</t>
   </si>
   <si>
-    <t>Name: "Short PW User", Phone: "9876543210", Email: "short_pw_1782125671330@example.com"</t>
+    <t>Name: "Short PW User", Phone: "9876543210", Email: "short_pw_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Error badge shows "Password should be at least 6 characters."</t>
@@ -737,7 +737,7 @@
     <t>Registration failure - Invalid phone format: abc</t>
   </si>
   <si>
-    <t>Name: "Bad Phone User", Phone: "abc", Email: "bad_phone_104_1782125671330@example.com"</t>
+    <t>Name: "Bad Phone User", Phone: "abc", Email: "bad_phone_104_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Error banner displayed or HTML5 blocks submission</t>
@@ -746,172 +746,172 @@
     <t>Registration failure - Invalid phone format: phone123</t>
   </si>
   <si>
-    <t>Name: "Bad Phone User", Phone: "phone123", Email: "bad_phone_105_1782125671330@example.com"</t>
+    <t>Name: "Bad Phone User", Phone: "phone123", Email: "bad_phone_105_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Registration failure - Invalid phone format: 9876abc123</t>
   </si>
   <si>
-    <t>Name: "Bad Phone User", Phone: "9876abc123", Email: "bad_phone_106_1782125671330@example.com"</t>
+    <t>Name: "Bad Phone User", Phone: "9876abc123", Email: "bad_phone_106_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Registration failure - Invalid phone format: 987654321a</t>
   </si>
   <si>
-    <t>Name: "Bad Phone User", Phone: "987654321a", Email: "bad_phone_107_1782125671330@example.com"</t>
+    <t>Name: "Bad Phone User", Phone: "987654321a", Email: "bad_phone_107_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Registration failure - Invalid phone format: !@#$%^&amp;*</t>
   </si>
   <si>
-    <t>Name: "Bad Phone User", Phone: "!@#$%^&amp;*", Email: "bad_phone_108_1782125671330@example.com"</t>
+    <t>Name: "Bad Phone User", Phone: "!@#$%^&amp;*", Email: "bad_phone_108_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Registration failure - Invalid phone format: 987654321!</t>
   </si>
   <si>
-    <t>Name: "Bad Phone User", Phone: "987654321!", Email: "bad_phone_109_1782125671330@example.com"</t>
+    <t>Name: "Bad Phone User", Phone: "987654321!", Email: "bad_phone_109_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Registration failure - Invalid phone format: 987654321_</t>
   </si>
   <si>
-    <t>Name: "Bad Phone User", Phone: "987654321_", Email: "bad_phone_110_1782125671330@example.com"</t>
+    <t>Name: "Bad Phone User", Phone: "987654321_", Email: "bad_phone_110_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Registration failure - Invalid phone format: @9876543</t>
   </si>
   <si>
-    <t>Name: "Bad Phone User", Phone: "@9876543", Email: "bad_phone_111_1782125671330@example.com"</t>
+    <t>Name: "Bad Phone User", Phone: "@9876543", Email: "bad_phone_111_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Registration failure - Invalid phone format: 98765#43</t>
   </si>
   <si>
-    <t>Name: "Bad Phone User", Phone: "98765#43", Email: "bad_phone_112_1782125671330@example.com"</t>
+    <t>Name: "Bad Phone User", Phone: "98765#43", Email: "bad_phone_112_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Registration failure - Invalid phone format: 1</t>
   </si>
   <si>
-    <t>Name: "Bad Phone User", Phone: "1", Email: "bad_phone_113_1782125671330@example.com"</t>
+    <t>Name: "Bad Phone User", Phone: "1", Email: "bad_phone_113_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Registration failure - Invalid phone format: 12</t>
   </si>
   <si>
-    <t>Name: "Bad Phone User", Phone: "12", Email: "bad_phone_114_1782125671330@example.com"</t>
+    <t>Name: "Bad Phone User", Phone: "12", Email: "bad_phone_114_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Registration failure - Invalid phone format: 123</t>
   </si>
   <si>
-    <t>Name: "Bad Phone User", Phone: "123", Email: "bad_phone_115_1782125671330@example.com"</t>
+    <t>Name: "Bad Phone User", Phone: "123", Email: "bad_phone_115_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Registration failure - Invalid phone format: 1234</t>
   </si>
   <si>
-    <t>Name: "Bad Phone User", Phone: "1234", Email: "bad_phone_116_1782125671330@example.com"</t>
+    <t>Name: "Bad Phone User", Phone: "1234", Email: "bad_phone_116_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Registration failure - Invalid phone format: 12345</t>
   </si>
   <si>
-    <t>Name: "Bad Phone User", Phone: "12345", Email: "bad_phone_117_1782125671330@example.com"</t>
+    <t>Name: "Bad Phone User", Phone: "12345", Email: "bad_phone_117_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Registration failure - Invalid phone format: 123456</t>
   </si>
   <si>
-    <t>Name: "Bad Phone User", Phone: "123456", Email: "bad_phone_118_1782125671330@example.com"</t>
+    <t>Name: "Bad Phone User", Phone: "123456", Email: "bad_phone_118_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Registration failure - Invalid phone format: 1234567890123456</t>
   </si>
   <si>
-    <t>Name: "Bad Phone User", Phone: "1234567890123456", Email: "bad_phone_119_1782125671330@example.com"</t>
+    <t>Name: "Bad Phone User", Phone: "1234567890123456", Email: "bad_phone_119_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Registration failure - Invalid phone format: 12345678901234567</t>
   </si>
   <si>
-    <t>Name: "Bad Phone User", Phone: "12345678901234567", Email: "bad_phone_120_1782125671330@example.com"</t>
+    <t>Name: "Bad Phone User", Phone: "12345678901234567", Email: "bad_phone_120_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Registration failure - Invalid phone format: 123456789012345678</t>
   </si>
   <si>
-    <t>Name: "Bad Phone User", Phone: "123456789012345678", Email: "bad_phone_121_1782125671330@example.com"</t>
+    <t>Name: "Bad Phone User", Phone: "123456789012345678", Email: "bad_phone_121_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Registration failure - Invalid phone format: 12345678901234567890</t>
   </si>
   <si>
-    <t>Name: "Bad Phone User", Phone: "12345678901234567890", Email: "bad_phone_122_1782125671330@example.com"</t>
+    <t>Name: "Bad Phone User", Phone: "12345678901234567890", Email: "bad_phone_122_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Registration failure - Invalid phone format: 123456789012345678901</t>
   </si>
   <si>
-    <t>Name: "Bad Phone User", Phone: "123456789012345678901", Email: "bad_phone_123_1782125671330@example.com"</t>
+    <t>Name: "Bad Phone User", Phone: "123456789012345678901", Email: "bad_phone_123_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Registration failure - Invalid phone format: 1234567890123456789012</t>
   </si>
   <si>
-    <t>Name: "Bad Phone User", Phone: "1234567890123456789012", Email: "bad_phone_124_1782125671330@example.com"</t>
+    <t>Name: "Bad Phone User", Phone: "1234567890123456789012", Email: "bad_phone_124_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Registration failure - Invalid phone format: bad</t>
   </si>
   <si>
-    <t>Name: "Bad Phone User", Phone: "bad", Email: "bad_phone_125_1782125671330@example.com"</t>
+    <t>Name: "Bad Phone User", Phone: "bad", Email: "bad_phone_125_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Registration failure - Invalid phone format: no-phone</t>
   </si>
   <si>
-    <t>Name: "Bad Phone User", Phone: "no-phone", Email: "bad_phone_126_1782125671330@example.com"</t>
+    <t>Name: "Bad Phone User", Phone: "no-phone", Email: "bad_phone_126_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Registration failure - Invalid phone format: number_one</t>
   </si>
   <si>
-    <t>Name: "Bad Phone User", Phone: "number_one", Email: "bad_phone_127_1782125671330@example.com"</t>
+    <t>Name: "Bad Phone User", Phone: "number_one", Email: "bad_phone_127_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Registration failure - Invalid phone format: digits!</t>
   </si>
   <si>
-    <t>Name: "Bad Phone User", Phone: "digits!", Email: "bad_phone_128_1782125671330@example.com"</t>
+    <t>Name: "Bad Phone User", Phone: "digits!", Email: "bad_phone_128_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Registration failure - Invalid phone format: ph-number</t>
   </si>
   <si>
-    <t>Name: "Bad Phone User", Phone: "ph-number", Email: "bad_phone_129_1782125671330@example.com"</t>
+    <t>Name: "Bad Phone User", Phone: "ph-number", Email: "bad_phone_129_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Registration failure - Invalid phone format: 12345a</t>
   </si>
   <si>
-    <t>Name: "Bad Phone User", Phone: "12345a", Email: "bad_phone_130_1782125671330@example.com"</t>
+    <t>Name: "Bad Phone User", Phone: "12345a", Email: "bad_phone_130_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Registration failure - Invalid phone format: 9876543210x</t>
   </si>
   <si>
-    <t>Name: "Bad Phone User", Phone: "9876543210x", Email: "bad_phone_131_1782125671330@example.com"</t>
+    <t>Name: "Bad Phone User", Phone: "9876543210x", Email: "bad_phone_131_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Registration failure - Invalid phone format: 0</t>
   </si>
   <si>
-    <t>Name: "Bad Phone User", Phone: "0", Email: "bad_phone_132_1782125671330@example.com"</t>
-  </si>
-  <si>
-    <t>Name: "Bad Phone User", Phone: "123", Email: "bad_phone_133_1782125671330@example.com"</t>
+    <t>Name: "Bad Phone User", Phone: "0", Email: "bad_phone_132_1782189503313@example.com"</t>
+  </si>
+  <si>
+    <t>Name: "Bad Phone User", Phone: "123", Email: "bad_phone_133_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Registration failure - Invalid email pattern format: reg_invalid_134_no_domain</t>
@@ -1124,55 +1124,55 @@
     <t>Registration boundary - Extreme lengths (Name: 250 chars, Email: 37 chars)</t>
   </si>
   <si>
-    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_168_1782125671330@example.com"</t>
-  </si>
-  <si>
-    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_170_1782125671330@example.com"</t>
-  </si>
-  <si>
-    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_172_1782125671330@example.com"</t>
-  </si>
-  <si>
-    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_174_1782125671330@example.com"</t>
-  </si>
-  <si>
-    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_176_1782125671330@example.com"</t>
-  </si>
-  <si>
-    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_178_1782125671330@example.com"</t>
-  </si>
-  <si>
-    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_180_1782125671330@example.com"</t>
-  </si>
-  <si>
-    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_182_1782125671330@example.com"</t>
-  </si>
-  <si>
-    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_184_1782125671330@example.com"</t>
-  </si>
-  <si>
-    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_186_1782125671330@example.com"</t>
-  </si>
-  <si>
-    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_188_1782125671330@example.com"</t>
-  </si>
-  <si>
-    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_190_1782125671330@example.com"</t>
-  </si>
-  <si>
-    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_192_1782125671330@example.com"</t>
-  </si>
-  <si>
-    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_194_1782125671330@example.com"</t>
-  </si>
-  <si>
-    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_196_1782125671330@example.com"</t>
-  </si>
-  <si>
-    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_198_1782125671330@example.com"</t>
-  </si>
-  <si>
-    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_200_1782125671330@example.com"</t>
+    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_168_1782189503313@example.com"</t>
+  </si>
+  <si>
+    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_170_1782189503313@example.com"</t>
+  </si>
+  <si>
+    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_172_1782189503313@example.com"</t>
+  </si>
+  <si>
+    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_174_1782189503313@example.com"</t>
+  </si>
+  <si>
+    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_176_1782189503313@example.com"</t>
+  </si>
+  <si>
+    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_178_1782189503313@example.com"</t>
+  </si>
+  <si>
+    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_180_1782189503313@example.com"</t>
+  </si>
+  <si>
+    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_182_1782189503313@example.com"</t>
+  </si>
+  <si>
+    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_184_1782189503313@example.com"</t>
+  </si>
+  <si>
+    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_186_1782189503313@example.com"</t>
+  </si>
+  <si>
+    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_188_1782189503313@example.com"</t>
+  </si>
+  <si>
+    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_190_1782189503313@example.com"</t>
+  </si>
+  <si>
+    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_192_1782189503313@example.com"</t>
+  </si>
+  <si>
+    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_194_1782189503313@example.com"</t>
+  </si>
+  <si>
+    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_196_1782189503313@example.com"</t>
+  </si>
+  <si>
+    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_198_1782189503313@example.com"</t>
+  </si>
+  <si>
+    <t>Name: "AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA", Phone: "9876543210", Email: "long_in_200_1782189503313@example.com"</t>
   </si>
   <si>
     <t>Emergency Suite</t>
@@ -2249,7 +2249,7 @@
         <v>18</v>
       </c>
       <c r="H7" s="7">
-        <v>12153</v>
+        <v>5614</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2275,7 +2275,7 @@
         <v>18</v>
       </c>
       <c r="H8" s="7">
-        <v>4032</v>
+        <v>13084</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2301,7 +2301,7 @@
         <v>18</v>
       </c>
       <c r="H9" s="7">
-        <v>4233</v>
+        <v>10722</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2327,7 +2327,7 @@
         <v>18</v>
       </c>
       <c r="H10" s="7">
-        <v>791</v>
+        <v>1368</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2353,7 +2353,7 @@
         <v>18</v>
       </c>
       <c r="H11" s="7">
-        <v>538</v>
+        <v>661</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2379,7 +2379,7 @@
         <v>18</v>
       </c>
       <c r="H12" s="7">
-        <v>494</v>
+        <v>760</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2405,7 +2405,7 @@
         <v>18</v>
       </c>
       <c r="H13" s="7">
-        <v>674</v>
+        <v>878</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2431,7 +2431,7 @@
         <v>18</v>
       </c>
       <c r="H14" s="7">
-        <v>563</v>
+        <v>842</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2457,7 +2457,7 @@
         <v>18</v>
       </c>
       <c r="H15" s="7">
-        <v>707</v>
+        <v>829</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2483,7 +2483,7 @@
         <v>18</v>
       </c>
       <c r="H16" s="7">
-        <v>574</v>
+        <v>710</v>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2509,7 +2509,7 @@
         <v>18</v>
       </c>
       <c r="H17" s="7">
-        <v>814</v>
+        <v>913</v>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2535,7 +2535,7 @@
         <v>18</v>
       </c>
       <c r="H18" s="7">
-        <v>560</v>
+        <v>714</v>
       </c>
     </row>
     <row r="19" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2561,7 +2561,7 @@
         <v>18</v>
       </c>
       <c r="H19" s="7">
-        <v>621</v>
+        <v>932</v>
       </c>
     </row>
     <row r="20" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2587,7 +2587,7 @@
         <v>18</v>
       </c>
       <c r="H20" s="7">
-        <v>549</v>
+        <v>592</v>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2613,7 +2613,7 @@
         <v>18</v>
       </c>
       <c r="H21" s="7">
-        <v>646</v>
+        <v>847</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2639,7 +2639,7 @@
         <v>18</v>
       </c>
       <c r="H22" s="7">
-        <v>552</v>
+        <v>557</v>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2665,7 +2665,7 @@
         <v>18</v>
       </c>
       <c r="H23" s="7">
-        <v>656</v>
+        <v>978</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2691,7 +2691,7 @@
         <v>18</v>
       </c>
       <c r="H24" s="7">
-        <v>668</v>
+        <v>815</v>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2717,7 +2717,7 @@
         <v>18</v>
       </c>
       <c r="H25" s="7">
-        <v>625</v>
+        <v>887</v>
       </c>
     </row>
     <row r="26" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2743,7 +2743,7 @@
         <v>18</v>
       </c>
       <c r="H26" s="7">
-        <v>527</v>
+        <v>793</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2769,7 +2769,7 @@
         <v>18</v>
       </c>
       <c r="H27" s="7">
-        <v>682</v>
+        <v>863</v>
       </c>
     </row>
     <row r="28" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2795,7 +2795,7 @@
         <v>18</v>
       </c>
       <c r="H28" s="7">
-        <v>566</v>
+        <v>718</v>
       </c>
     </row>
     <row r="29" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2821,7 +2821,7 @@
         <v>18</v>
       </c>
       <c r="H29" s="7">
-        <v>658</v>
+        <v>779</v>
       </c>
     </row>
     <row r="30" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2847,7 +2847,7 @@
         <v>18</v>
       </c>
       <c r="H30" s="7">
-        <v>627</v>
+        <v>723</v>
       </c>
     </row>
     <row r="31" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2873,7 +2873,7 @@
         <v>18</v>
       </c>
       <c r="H31" s="7">
-        <v>708</v>
+        <v>943</v>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2899,7 +2899,7 @@
         <v>18</v>
       </c>
       <c r="H32" s="7">
-        <v>552</v>
+        <v>1084</v>
       </c>
     </row>
     <row r="33" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2925,7 +2925,7 @@
         <v>18</v>
       </c>
       <c r="H33" s="7">
-        <v>649</v>
+        <v>975</v>
       </c>
     </row>
     <row r="34" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2951,7 +2951,7 @@
         <v>18</v>
       </c>
       <c r="H34" s="7">
-        <v>609</v>
+        <v>980</v>
       </c>
     </row>
     <row r="35" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2977,7 +2977,7 @@
         <v>18</v>
       </c>
       <c r="H35" s="7">
-        <v>626</v>
+        <v>849</v>
       </c>
     </row>
     <row r="36" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3003,7 +3003,7 @@
         <v>18</v>
       </c>
       <c r="H36" s="7">
-        <v>586</v>
+        <v>639</v>
       </c>
     </row>
     <row r="37" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3029,7 +3029,7 @@
         <v>18</v>
       </c>
       <c r="H37" s="7">
-        <v>633</v>
+        <v>993</v>
       </c>
     </row>
     <row r="38" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3055,7 +3055,7 @@
         <v>18</v>
       </c>
       <c r="H38" s="7">
-        <v>582</v>
+        <v>665</v>
       </c>
     </row>
     <row r="39" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3081,7 +3081,7 @@
         <v>18</v>
       </c>
       <c r="H39" s="7">
-        <v>738</v>
+        <v>1108</v>
       </c>
     </row>
     <row r="40" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3107,7 +3107,7 @@
         <v>18</v>
       </c>
       <c r="H40" s="7">
-        <v>594</v>
+        <v>816</v>
       </c>
     </row>
     <row r="41" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3133,7 +3133,7 @@
         <v>18</v>
       </c>
       <c r="H41" s="7">
-        <v>691</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="42" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3159,7 +3159,7 @@
         <v>18</v>
       </c>
       <c r="H42" s="7">
-        <v>660</v>
+        <v>811</v>
       </c>
     </row>
     <row r="43" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3185,7 +3185,7 @@
         <v>18</v>
       </c>
       <c r="H43" s="7">
-        <v>676</v>
+        <v>795</v>
       </c>
     </row>
     <row r="44" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3211,7 +3211,7 @@
         <v>18</v>
       </c>
       <c r="H44" s="7">
-        <v>572</v>
+        <v>942</v>
       </c>
     </row>
     <row r="45" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3237,7 +3237,7 @@
         <v>18</v>
       </c>
       <c r="H45" s="7">
-        <v>654</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="46" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3263,7 +3263,7 @@
         <v>18</v>
       </c>
       <c r="H46" s="7">
-        <v>540</v>
+        <v>943</v>
       </c>
     </row>
     <row r="47" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3289,7 +3289,7 @@
         <v>18</v>
       </c>
       <c r="H47" s="7">
-        <v>662</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="48" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3315,7 +3315,7 @@
         <v>18</v>
       </c>
       <c r="H48" s="7">
-        <v>570</v>
+        <v>1103</v>
       </c>
     </row>
     <row r="49" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3341,7 +3341,7 @@
         <v>18</v>
       </c>
       <c r="H49" s="7">
-        <v>662</v>
+        <v>840</v>
       </c>
     </row>
     <row r="50" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3367,7 +3367,7 @@
         <v>18</v>
       </c>
       <c r="H50" s="7">
-        <v>563</v>
+        <v>915</v>
       </c>
     </row>
     <row r="51" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3393,7 +3393,7 @@
         <v>18</v>
       </c>
       <c r="H51" s="7">
-        <v>679</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="52" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3419,7 +3419,7 @@
         <v>18</v>
       </c>
       <c r="H52" s="7">
-        <v>592</v>
+        <v>848</v>
       </c>
     </row>
     <row r="53" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3445,7 +3445,7 @@
         <v>18</v>
       </c>
       <c r="H53" s="7">
-        <v>709</v>
+        <v>843</v>
       </c>
     </row>
     <row r="54" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3471,7 +3471,7 @@
         <v>18</v>
       </c>
       <c r="H54" s="7">
-        <v>729</v>
+        <v>727</v>
       </c>
     </row>
     <row r="55" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3497,7 +3497,7 @@
         <v>18</v>
       </c>
       <c r="H55" s="7">
-        <v>640</v>
+        <v>814</v>
       </c>
     </row>
     <row r="56" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3523,7 +3523,7 @@
         <v>18</v>
       </c>
       <c r="H56" s="7">
-        <v>576</v>
+        <v>663</v>
       </c>
     </row>
     <row r="57" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3549,7 +3549,7 @@
         <v>18</v>
       </c>
       <c r="H57" s="7">
-        <v>579</v>
+        <v>774</v>
       </c>
     </row>
     <row r="58" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3575,7 +3575,7 @@
         <v>18</v>
       </c>
       <c r="H58" s="7">
-        <v>1831</v>
+        <v>898</v>
       </c>
     </row>
     <row r="59" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3601,7 +3601,7 @@
         <v>18</v>
       </c>
       <c r="H59" s="7">
-        <v>597</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="60" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3627,7 +3627,7 @@
         <v>18</v>
       </c>
       <c r="H60" s="7">
-        <v>602</v>
+        <v>881</v>
       </c>
     </row>
     <row r="61" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3653,7 +3653,7 @@
         <v>18</v>
       </c>
       <c r="H61" s="7">
-        <v>577</v>
+        <v>932</v>
       </c>
     </row>
     <row r="62" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3679,7 +3679,7 @@
         <v>18</v>
       </c>
       <c r="H62" s="7">
-        <v>1440</v>
+        <v>1453</v>
       </c>
     </row>
     <row r="63" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3705,7 +3705,7 @@
         <v>18</v>
       </c>
       <c r="H63" s="7">
-        <v>654</v>
+        <v>760</v>
       </c>
     </row>
     <row r="64" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3731,7 +3731,7 @@
         <v>18</v>
       </c>
       <c r="H64" s="7">
-        <v>631</v>
+        <v>984</v>
       </c>
     </row>
     <row r="65" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3757,7 +3757,7 @@
         <v>18</v>
       </c>
       <c r="H65" s="7">
-        <v>601</v>
+        <v>589</v>
       </c>
     </row>
     <row r="66" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3783,7 +3783,7 @@
         <v>18</v>
       </c>
       <c r="H66" s="7">
-        <v>642</v>
+        <v>1101</v>
       </c>
     </row>
     <row r="67" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3809,7 +3809,7 @@
         <v>18</v>
       </c>
       <c r="H67" s="7">
-        <v>618</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="68" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3835,7 +3835,7 @@
         <v>18</v>
       </c>
       <c r="H68" s="7">
-        <v>619</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="69" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3861,7 +3861,7 @@
         <v>18</v>
       </c>
       <c r="H69" s="7">
-        <v>604</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="70" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3887,7 +3887,7 @@
         <v>18</v>
       </c>
       <c r="H70" s="7">
-        <v>568</v>
+        <v>899</v>
       </c>
     </row>
     <row r="71" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3913,7 +3913,7 @@
         <v>18</v>
       </c>
       <c r="H71" s="7">
-        <v>674</v>
+        <v>962</v>
       </c>
     </row>
     <row r="72" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3939,7 +3939,7 @@
         <v>18</v>
       </c>
       <c r="H72" s="7">
-        <v>560</v>
+        <v>816</v>
       </c>
     </row>
     <row r="73" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3965,7 +3965,7 @@
         <v>18</v>
       </c>
       <c r="H73" s="7">
-        <v>609</v>
+        <v>868</v>
       </c>
     </row>
     <row r="74" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -3991,7 +3991,7 @@
         <v>18</v>
       </c>
       <c r="H74" s="7">
-        <v>604</v>
+        <v>932</v>
       </c>
     </row>
     <row r="75" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4017,7 +4017,7 @@
         <v>18</v>
       </c>
       <c r="H75" s="7">
-        <v>591</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="76" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4043,7 +4043,7 @@
         <v>18</v>
       </c>
       <c r="H76" s="7">
-        <v>571</v>
+        <v>867</v>
       </c>
     </row>
     <row r="77" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4069,7 +4069,7 @@
         <v>18</v>
       </c>
       <c r="H77" s="7">
-        <v>602</v>
+        <v>759</v>
       </c>
     </row>
     <row r="78" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4095,7 +4095,7 @@
         <v>18</v>
       </c>
       <c r="H78" s="7">
-        <v>602</v>
+        <v>834</v>
       </c>
     </row>
     <row r="79" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4121,7 +4121,7 @@
         <v>18</v>
       </c>
       <c r="H79" s="7">
-        <v>585</v>
+        <v>789</v>
       </c>
     </row>
     <row r="80" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4147,7 +4147,7 @@
         <v>18</v>
       </c>
       <c r="H80" s="7">
-        <v>640</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="81" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4173,7 +4173,7 @@
         <v>18</v>
       </c>
       <c r="H81" s="7">
-        <v>600</v>
+        <v>952</v>
       </c>
     </row>
     <row r="82" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4199,7 +4199,7 @@
         <v>18</v>
       </c>
       <c r="H82" s="7">
-        <v>2336</v>
+        <v>3764</v>
       </c>
     </row>
     <row r="83" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4225,7 +4225,7 @@
         <v>18</v>
       </c>
       <c r="H83" s="7">
-        <v>2200</v>
+        <v>3238</v>
       </c>
     </row>
     <row r="84" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4251,7 +4251,7 @@
         <v>18</v>
       </c>
       <c r="H84" s="7">
-        <v>2225</v>
+        <v>3621</v>
       </c>
     </row>
     <row r="85" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4277,7 +4277,7 @@
         <v>18</v>
       </c>
       <c r="H85" s="7">
-        <v>2231</v>
+        <v>3705</v>
       </c>
     </row>
     <row r="86" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4303,7 +4303,7 @@
         <v>18</v>
       </c>
       <c r="H86" s="7">
-        <v>2215</v>
+        <v>3505</v>
       </c>
     </row>
     <row r="87" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4329,7 +4329,7 @@
         <v>18</v>
       </c>
       <c r="H87" s="7">
-        <v>2298</v>
+        <v>3513</v>
       </c>
     </row>
     <row r="88" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4355,7 +4355,7 @@
         <v>18</v>
       </c>
       <c r="H88" s="7">
-        <v>2226</v>
+        <v>4101</v>
       </c>
     </row>
     <row r="89" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4381,7 +4381,7 @@
         <v>18</v>
       </c>
       <c r="H89" s="7">
-        <v>2298</v>
+        <v>3805</v>
       </c>
     </row>
     <row r="90" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4407,7 +4407,7 @@
         <v>18</v>
       </c>
       <c r="H90" s="7">
-        <v>2269</v>
+        <v>4865</v>
       </c>
     </row>
     <row r="91" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4433,7 +4433,7 @@
         <v>18</v>
       </c>
       <c r="H91" s="7">
-        <v>2352</v>
+        <v>5097</v>
       </c>
     </row>
     <row r="92" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4459,7 +4459,7 @@
         <v>18</v>
       </c>
       <c r="H92" s="7">
-        <v>2313</v>
+        <v>5015</v>
       </c>
     </row>
     <row r="93" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4485,7 +4485,7 @@
         <v>18</v>
       </c>
       <c r="H93" s="7">
-        <v>2375</v>
+        <v>4593</v>
       </c>
     </row>
     <row r="94" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4511,7 +4511,7 @@
         <v>18</v>
       </c>
       <c r="H94" s="7">
-        <v>2354</v>
+        <v>5008</v>
       </c>
     </row>
     <row r="95" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4537,7 +4537,7 @@
         <v>18</v>
       </c>
       <c r="H95" s="7">
-        <v>2325</v>
+        <v>4764</v>
       </c>
     </row>
     <row r="96" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4563,7 +4563,7 @@
         <v>18</v>
       </c>
       <c r="H96" s="7">
-        <v>2402</v>
+        <v>5573</v>
       </c>
     </row>
     <row r="97" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4589,7 +4589,7 @@
         <v>18</v>
       </c>
       <c r="H97" s="7">
-        <v>2400</v>
+        <v>4858</v>
       </c>
     </row>
     <row r="98" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4615,7 +4615,7 @@
         <v>18</v>
       </c>
       <c r="H98" s="7">
-        <v>2441</v>
+        <v>5557</v>
       </c>
     </row>
     <row r="99" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4641,7 +4641,7 @@
         <v>18</v>
       </c>
       <c r="H99" s="7">
-        <v>2536</v>
+        <v>5318</v>
       </c>
     </row>
     <row r="100" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4667,7 +4667,7 @@
         <v>18</v>
       </c>
       <c r="H100" s="7">
-        <v>2394</v>
+        <v>5002</v>
       </c>
     </row>
     <row r="101" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4693,7 +4693,7 @@
         <v>18</v>
       </c>
       <c r="H101" s="7">
-        <v>2511</v>
+        <v>6674</v>
       </c>
     </row>
     <row r="102" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4719,7 +4719,7 @@
         <v>18</v>
       </c>
       <c r="H102" s="7">
-        <v>2491</v>
+        <v>6527</v>
       </c>
     </row>
     <row r="103" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4745,7 +4745,7 @@
         <v>18</v>
       </c>
       <c r="H103" s="7">
-        <v>2519</v>
+        <v>6287</v>
       </c>
     </row>
     <row r="104" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4771,7 +4771,7 @@
         <v>18</v>
       </c>
       <c r="H104" s="7">
-        <v>2592</v>
+        <v>6636</v>
       </c>
     </row>
     <row r="105" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4797,7 +4797,7 @@
         <v>18</v>
       </c>
       <c r="H105" s="7">
-        <v>2585</v>
+        <v>7329</v>
       </c>
     </row>
     <row r="106" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4823,7 +4823,7 @@
         <v>18</v>
       </c>
       <c r="H106" s="7">
-        <v>2626</v>
+        <v>5447</v>
       </c>
     </row>
     <row r="107" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4849,7 +4849,7 @@
         <v>18</v>
       </c>
       <c r="H107" s="7">
-        <v>4331</v>
+        <v>5298</v>
       </c>
     </row>
     <row r="108" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4875,7 +4875,7 @@
         <v>18</v>
       </c>
       <c r="H108" s="7">
-        <v>1215</v>
+        <v>1898</v>
       </c>
     </row>
     <row r="109" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4901,7 +4901,7 @@
         <v>18</v>
       </c>
       <c r="H109" s="7">
-        <v>923</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="110" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4927,7 +4927,7 @@
         <v>18</v>
       </c>
       <c r="H110" s="7">
-        <v>1035</v>
+        <v>1752</v>
       </c>
     </row>
     <row r="111" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4953,7 +4953,7 @@
         <v>18</v>
       </c>
       <c r="H111" s="7">
-        <v>1060</v>
+        <v>1830</v>
       </c>
     </row>
     <row r="112" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -4979,7 +4979,7 @@
         <v>18</v>
       </c>
       <c r="H112" s="7">
-        <v>990</v>
+        <v>2083</v>
       </c>
     </row>
     <row r="113" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5005,7 +5005,7 @@
         <v>18</v>
       </c>
       <c r="H113" s="7">
-        <v>1057</v>
+        <v>2156</v>
       </c>
     </row>
     <row r="114" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5031,7 +5031,7 @@
         <v>18</v>
       </c>
       <c r="H114" s="7">
-        <v>1078</v>
+        <v>1732</v>
       </c>
     </row>
     <row r="115" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5057,7 +5057,7 @@
         <v>18</v>
       </c>
       <c r="H115" s="7">
-        <v>1051</v>
+        <v>1932</v>
       </c>
     </row>
     <row r="116" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5083,7 +5083,7 @@
         <v>18</v>
       </c>
       <c r="H116" s="7">
-        <v>1081</v>
+        <v>1834</v>
       </c>
     </row>
     <row r="117" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5109,7 +5109,7 @@
         <v>18</v>
       </c>
       <c r="H117" s="7">
-        <v>987</v>
+        <v>1754</v>
       </c>
     </row>
     <row r="118" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5135,7 +5135,7 @@
         <v>18</v>
       </c>
       <c r="H118" s="7">
-        <v>1109</v>
+        <v>1709</v>
       </c>
     </row>
     <row r="119" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5161,7 +5161,7 @@
         <v>18</v>
       </c>
       <c r="H119" s="7">
-        <v>962</v>
+        <v>1496</v>
       </c>
     </row>
     <row r="120" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5187,7 +5187,7 @@
         <v>18</v>
       </c>
       <c r="H120" s="7">
-        <v>952</v>
+        <v>2084</v>
       </c>
     </row>
     <row r="121" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5213,7 +5213,7 @@
         <v>18</v>
       </c>
       <c r="H121" s="7">
-        <v>1031</v>
+        <v>1882</v>
       </c>
     </row>
     <row r="122" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5239,7 +5239,7 @@
         <v>18</v>
       </c>
       <c r="H122" s="7">
-        <v>1028</v>
+        <v>1987</v>
       </c>
     </row>
     <row r="123" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5265,7 +5265,7 @@
         <v>18</v>
       </c>
       <c r="H123" s="7">
-        <v>998</v>
+        <v>1878</v>
       </c>
     </row>
     <row r="124" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5291,7 +5291,7 @@
         <v>18</v>
       </c>
       <c r="H124" s="7">
-        <v>984</v>
+        <v>2166</v>
       </c>
     </row>
     <row r="125" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5317,7 +5317,7 @@
         <v>18</v>
       </c>
       <c r="H125" s="7">
-        <v>1033</v>
+        <v>2173</v>
       </c>
     </row>
     <row r="126" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5343,7 +5343,7 @@
         <v>18</v>
       </c>
       <c r="H126" s="7">
-        <v>1007</v>
+        <v>2012</v>
       </c>
     </row>
     <row r="127" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5369,7 +5369,7 @@
         <v>18</v>
       </c>
       <c r="H127" s="7">
-        <v>1064</v>
+        <v>1902</v>
       </c>
     </row>
     <row r="128" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5395,7 +5395,7 @@
         <v>18</v>
       </c>
       <c r="H128" s="7">
-        <v>1079</v>
+        <v>2093</v>
       </c>
     </row>
     <row r="129" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5421,7 +5421,7 @@
         <v>18</v>
       </c>
       <c r="H129" s="7">
-        <v>1076</v>
+        <v>1897</v>
       </c>
     </row>
     <row r="130" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5447,7 +5447,7 @@
         <v>18</v>
       </c>
       <c r="H130" s="7">
-        <v>1093</v>
+        <v>1830</v>
       </c>
     </row>
     <row r="131" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5473,7 +5473,7 @@
         <v>18</v>
       </c>
       <c r="H131" s="7">
-        <v>1001</v>
+        <v>1951</v>
       </c>
     </row>
     <row r="132" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5499,7 +5499,7 @@
         <v>18</v>
       </c>
       <c r="H132" s="7">
-        <v>1087</v>
+        <v>2383</v>
       </c>
     </row>
     <row r="133" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5525,7 +5525,7 @@
         <v>18</v>
       </c>
       <c r="H133" s="7">
-        <v>1017</v>
+        <v>2114</v>
       </c>
     </row>
     <row r="134" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5551,7 +5551,7 @@
         <v>18</v>
       </c>
       <c r="H134" s="7">
-        <v>1102</v>
+        <v>1948</v>
       </c>
     </row>
     <row r="135" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5577,7 +5577,7 @@
         <v>18</v>
       </c>
       <c r="H135" s="7">
-        <v>1090</v>
+        <v>1857</v>
       </c>
     </row>
     <row r="136" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5603,7 +5603,7 @@
         <v>18</v>
       </c>
       <c r="H136" s="7">
-        <v>989</v>
+        <v>2098</v>
       </c>
     </row>
     <row r="137" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5629,7 +5629,7 @@
         <v>18</v>
       </c>
       <c r="H137" s="7">
-        <v>1035</v>
+        <v>1950</v>
       </c>
     </row>
     <row r="138" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5655,7 +5655,7 @@
         <v>18</v>
       </c>
       <c r="H138" s="7">
-        <v>1052</v>
+        <v>1779</v>
       </c>
     </row>
     <row r="139" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5681,7 +5681,7 @@
         <v>18</v>
       </c>
       <c r="H139" s="7">
-        <v>1010</v>
+        <v>2053</v>
       </c>
     </row>
     <row r="140" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5707,7 +5707,7 @@
         <v>18</v>
       </c>
       <c r="H140" s="7">
-        <v>999</v>
+        <v>2015</v>
       </c>
     </row>
     <row r="141" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5733,7 +5733,7 @@
         <v>18</v>
       </c>
       <c r="H141" s="7">
-        <v>955</v>
+        <v>1758</v>
       </c>
     </row>
     <row r="142" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5759,7 +5759,7 @@
         <v>18</v>
       </c>
       <c r="H142" s="7">
-        <v>983</v>
+        <v>1775</v>
       </c>
     </row>
     <row r="143" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5785,7 +5785,7 @@
         <v>18</v>
       </c>
       <c r="H143" s="7">
-        <v>1006</v>
+        <v>1738</v>
       </c>
     </row>
     <row r="144" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5811,7 +5811,7 @@
         <v>18</v>
       </c>
       <c r="H144" s="7">
-        <v>909</v>
+        <v>1729</v>
       </c>
     </row>
     <row r="145" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5837,7 +5837,7 @@
         <v>18</v>
       </c>
       <c r="H145" s="7">
-        <v>931</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="146" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5863,7 +5863,7 @@
         <v>18</v>
       </c>
       <c r="H146" s="7">
-        <v>883</v>
+        <v>1617</v>
       </c>
     </row>
     <row r="147" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5889,7 +5889,7 @@
         <v>18</v>
       </c>
       <c r="H147" s="7">
-        <v>944</v>
+        <v>2063</v>
       </c>
     </row>
     <row r="148" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5915,7 +5915,7 @@
         <v>18</v>
       </c>
       <c r="H148" s="7">
-        <v>995</v>
+        <v>1627</v>
       </c>
     </row>
     <row r="149" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5941,7 +5941,7 @@
         <v>18</v>
       </c>
       <c r="H149" s="7">
-        <v>925</v>
+        <v>1981</v>
       </c>
     </row>
     <row r="150" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5967,7 +5967,7 @@
         <v>18</v>
       </c>
       <c r="H150" s="7">
-        <v>929</v>
+        <v>1847</v>
       </c>
     </row>
     <row r="151" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -5993,7 +5993,7 @@
         <v>18</v>
       </c>
       <c r="H151" s="7">
-        <v>948</v>
+        <v>1781</v>
       </c>
     </row>
     <row r="152" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6019,7 +6019,7 @@
         <v>18</v>
       </c>
       <c r="H152" s="7">
-        <v>938</v>
+        <v>1758</v>
       </c>
     </row>
     <row r="153" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6045,7 +6045,7 @@
         <v>18</v>
       </c>
       <c r="H153" s="7">
-        <v>933</v>
+        <v>1898</v>
       </c>
     </row>
     <row r="154" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6071,7 +6071,7 @@
         <v>18</v>
       </c>
       <c r="H154" s="7">
-        <v>954</v>
+        <v>1522</v>
       </c>
     </row>
     <row r="155" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6097,7 +6097,7 @@
         <v>18</v>
       </c>
       <c r="H155" s="7">
-        <v>933</v>
+        <v>1532</v>
       </c>
     </row>
     <row r="156" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6123,7 +6123,7 @@
         <v>18</v>
       </c>
       <c r="H156" s="7">
-        <v>971</v>
+        <v>1604</v>
       </c>
     </row>
     <row r="157" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6149,7 +6149,7 @@
         <v>18</v>
       </c>
       <c r="H157" s="7">
-        <v>1011</v>
+        <v>1498</v>
       </c>
     </row>
     <row r="158" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6175,7 +6175,7 @@
         <v>18</v>
       </c>
       <c r="H158" s="7">
-        <v>938</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="159" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6201,7 +6201,7 @@
         <v>18</v>
       </c>
       <c r="H159" s="7">
-        <v>943</v>
+        <v>1741</v>
       </c>
     </row>
     <row r="160" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6227,7 +6227,7 @@
         <v>18</v>
       </c>
       <c r="H160" s="7">
-        <v>924</v>
+        <v>1739</v>
       </c>
     </row>
     <row r="161" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6253,7 +6253,7 @@
         <v>18</v>
       </c>
       <c r="H161" s="7">
-        <v>910</v>
+        <v>1822</v>
       </c>
     </row>
     <row r="162" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6279,7 +6279,7 @@
         <v>18</v>
       </c>
       <c r="H162" s="7">
-        <v>920</v>
+        <v>1641</v>
       </c>
     </row>
     <row r="163" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6305,7 +6305,7 @@
         <v>18</v>
       </c>
       <c r="H163" s="7">
-        <v>994</v>
+        <v>1741</v>
       </c>
     </row>
     <row r="164" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6331,7 +6331,7 @@
         <v>18</v>
       </c>
       <c r="H164" s="7">
-        <v>1003</v>
+        <v>1734</v>
       </c>
     </row>
     <row r="165" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6357,7 +6357,7 @@
         <v>18</v>
       </c>
       <c r="H165" s="7">
-        <v>960</v>
+        <v>2013</v>
       </c>
     </row>
     <row r="166" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6383,7 +6383,7 @@
         <v>18</v>
       </c>
       <c r="H166" s="7">
-        <v>926</v>
+        <v>2123</v>
       </c>
     </row>
     <row r="167" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6409,7 +6409,7 @@
         <v>18</v>
       </c>
       <c r="H167" s="7">
-        <v>946</v>
+        <v>2157</v>
       </c>
     </row>
     <row r="168" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6435,7 +6435,7 @@
         <v>18</v>
       </c>
       <c r="H168" s="7">
-        <v>935</v>
+        <v>1829</v>
       </c>
     </row>
     <row r="169" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6461,7 +6461,7 @@
         <v>18</v>
       </c>
       <c r="H169" s="7">
-        <v>937</v>
+        <v>1682</v>
       </c>
     </row>
     <row r="170" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6487,7 +6487,7 @@
         <v>18</v>
       </c>
       <c r="H170" s="7">
-        <v>968</v>
+        <v>1904</v>
       </c>
     </row>
     <row r="171" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6513,7 +6513,7 @@
         <v>18</v>
       </c>
       <c r="H171" s="7">
-        <v>970</v>
+        <v>1890</v>
       </c>
     </row>
     <row r="172" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6539,7 +6539,7 @@
         <v>18</v>
       </c>
       <c r="H172" s="7">
-        <v>942</v>
+        <v>1639</v>
       </c>
     </row>
     <row r="173" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6565,7 +6565,7 @@
         <v>18</v>
       </c>
       <c r="H173" s="7">
-        <v>1498</v>
+        <v>3095</v>
       </c>
     </row>
     <row r="174" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6591,7 +6591,7 @@
         <v>18</v>
       </c>
       <c r="H174" s="7">
-        <v>1732</v>
+        <v>3660</v>
       </c>
     </row>
     <row r="175" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6617,7 +6617,7 @@
         <v>18</v>
       </c>
       <c r="H175" s="7">
-        <v>1488</v>
+        <v>3521</v>
       </c>
     </row>
     <row r="176" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6643,7 +6643,7 @@
         <v>18</v>
       </c>
       <c r="H176" s="7">
-        <v>1743</v>
+        <v>3641</v>
       </c>
     </row>
     <row r="177" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6669,7 +6669,7 @@
         <v>18</v>
       </c>
       <c r="H177" s="7">
-        <v>1545</v>
+        <v>3085</v>
       </c>
     </row>
     <row r="178" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6695,7 +6695,7 @@
         <v>18</v>
       </c>
       <c r="H178" s="7">
-        <v>1661</v>
+        <v>3314</v>
       </c>
     </row>
     <row r="179" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6721,7 +6721,7 @@
         <v>18</v>
       </c>
       <c r="H179" s="7">
-        <v>1504</v>
+        <v>2996</v>
       </c>
     </row>
     <row r="180" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6747,7 +6747,7 @@
         <v>18</v>
       </c>
       <c r="H180" s="7">
-        <v>1696</v>
+        <v>3723</v>
       </c>
     </row>
     <row r="181" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6773,7 +6773,7 @@
         <v>18</v>
       </c>
       <c r="H181" s="7">
-        <v>1609</v>
+        <v>2826</v>
       </c>
     </row>
     <row r="182" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6799,7 +6799,7 @@
         <v>18</v>
       </c>
       <c r="H182" s="7">
-        <v>1758</v>
+        <v>2914</v>
       </c>
     </row>
     <row r="183" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6825,7 +6825,7 @@
         <v>18</v>
       </c>
       <c r="H183" s="7">
-        <v>1559</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="184" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6851,7 +6851,7 @@
         <v>18</v>
       </c>
       <c r="H184" s="7">
-        <v>1699</v>
+        <v>3536</v>
       </c>
     </row>
     <row r="185" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6877,7 +6877,7 @@
         <v>18</v>
       </c>
       <c r="H185" s="7">
-        <v>1460</v>
+        <v>3144</v>
       </c>
     </row>
     <row r="186" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6903,7 +6903,7 @@
         <v>18</v>
       </c>
       <c r="H186" s="7">
-        <v>1646</v>
+        <v>3567</v>
       </c>
     </row>
     <row r="187" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6929,7 +6929,7 @@
         <v>18</v>
       </c>
       <c r="H187" s="7">
-        <v>1575</v>
+        <v>2821</v>
       </c>
     </row>
     <row r="188" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6955,7 +6955,7 @@
         <v>18</v>
       </c>
       <c r="H188" s="7">
-        <v>1585</v>
+        <v>3155</v>
       </c>
     </row>
     <row r="189" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -6981,7 +6981,7 @@
         <v>18</v>
       </c>
       <c r="H189" s="7">
-        <v>1449</v>
+        <v>3124</v>
       </c>
     </row>
     <row r="190" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7007,7 +7007,7 @@
         <v>18</v>
       </c>
       <c r="H190" s="7">
-        <v>1597</v>
+        <v>2088</v>
       </c>
     </row>
     <row r="191" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7033,7 +7033,7 @@
         <v>18</v>
       </c>
       <c r="H191" s="7">
-        <v>1458</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="192" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7059,7 +7059,7 @@
         <v>18</v>
       </c>
       <c r="H192" s="7">
-        <v>1705</v>
+        <v>2348</v>
       </c>
     </row>
     <row r="193" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7085,7 +7085,7 @@
         <v>18</v>
       </c>
       <c r="H193" s="7">
-        <v>1513</v>
+        <v>2073</v>
       </c>
     </row>
     <row r="194" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7111,7 +7111,7 @@
         <v>18</v>
       </c>
       <c r="H194" s="7">
-        <v>1720</v>
+        <v>3242</v>
       </c>
     </row>
     <row r="195" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7137,7 +7137,7 @@
         <v>18</v>
       </c>
       <c r="H195" s="7">
-        <v>1500</v>
+        <v>2772</v>
       </c>
     </row>
     <row r="196" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7163,7 +7163,7 @@
         <v>18</v>
       </c>
       <c r="H196" s="7">
-        <v>1614</v>
+        <v>3033</v>
       </c>
     </row>
     <row r="197" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7189,7 +7189,7 @@
         <v>18</v>
       </c>
       <c r="H197" s="7">
-        <v>1490</v>
+        <v>2873</v>
       </c>
     </row>
     <row r="198" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7215,7 +7215,7 @@
         <v>18</v>
       </c>
       <c r="H198" s="7">
-        <v>1603</v>
+        <v>3231</v>
       </c>
     </row>
     <row r="199" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7241,7 +7241,7 @@
         <v>18</v>
       </c>
       <c r="H199" s="7">
-        <v>1449</v>
+        <v>3059</v>
       </c>
     </row>
     <row r="200" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7267,7 +7267,7 @@
         <v>18</v>
       </c>
       <c r="H200" s="7">
-        <v>1582</v>
+        <v>3724</v>
       </c>
     </row>
     <row r="201" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7293,7 +7293,7 @@
         <v>18</v>
       </c>
       <c r="H201" s="7">
-        <v>1416</v>
+        <v>3280</v>
       </c>
     </row>
     <row r="202" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7319,7 +7319,7 @@
         <v>18</v>
       </c>
       <c r="H202" s="7">
-        <v>1561</v>
+        <v>3081</v>
       </c>
     </row>
     <row r="203" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7345,7 +7345,7 @@
         <v>18</v>
       </c>
       <c r="H203" s="7">
-        <v>1418</v>
+        <v>2796</v>
       </c>
     </row>
     <row r="204" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7371,7 +7371,7 @@
         <v>18</v>
       </c>
       <c r="H204" s="7">
-        <v>1590</v>
+        <v>3187</v>
       </c>
     </row>
     <row r="205" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7397,7 +7397,7 @@
         <v>18</v>
       </c>
       <c r="H205" s="7">
-        <v>1468</v>
+        <v>3004</v>
       </c>
     </row>
     <row r="206" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7423,7 +7423,7 @@
         <v>18</v>
       </c>
       <c r="H206" s="7">
-        <v>1710</v>
+        <v>3470</v>
       </c>
     </row>
     <row r="207" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7449,7 +7449,7 @@
         <v>18</v>
       </c>
       <c r="H207" s="7">
-        <v>1907</v>
+        <v>2720</v>
       </c>
     </row>
     <row r="208" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7475,7 +7475,7 @@
         <v>18</v>
       </c>
       <c r="H208" s="7">
-        <v>1258</v>
+        <v>2016</v>
       </c>
     </row>
     <row r="209" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7501,7 +7501,7 @@
         <v>18</v>
       </c>
       <c r="H209" s="7">
-        <v>1055</v>
+        <v>1612</v>
       </c>
     </row>
     <row r="210" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7527,7 +7527,7 @@
         <v>18</v>
       </c>
       <c r="H210" s="7">
-        <v>1216</v>
+        <v>1937</v>
       </c>
     </row>
     <row r="211" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7553,7 +7553,7 @@
         <v>18</v>
       </c>
       <c r="H211" s="7">
-        <v>1260</v>
+        <v>1955</v>
       </c>
     </row>
     <row r="212" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7579,7 +7579,7 @@
         <v>18</v>
       </c>
       <c r="H212" s="7">
-        <v>4485</v>
+        <v>5373</v>
       </c>
     </row>
     <row r="213" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7605,7 +7605,7 @@
         <v>18</v>
       </c>
       <c r="H213" s="7">
-        <v>4588</v>
+        <v>5320</v>
       </c>
     </row>
     <row r="214" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7631,7 +7631,7 @@
         <v>18</v>
       </c>
       <c r="H214" s="7">
-        <v>4546</v>
+        <v>5307</v>
       </c>
     </row>
     <row r="215" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7657,7 +7657,7 @@
         <v>18</v>
       </c>
       <c r="H215" s="7">
-        <v>4563</v>
+        <v>5049</v>
       </c>
     </row>
     <row r="216" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7683,7 +7683,7 @@
         <v>18</v>
       </c>
       <c r="H216" s="7">
-        <v>2857</v>
+        <v>2966</v>
       </c>
     </row>
     <row r="217" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7709,7 +7709,7 @@
         <v>18</v>
       </c>
       <c r="H217" s="7">
-        <v>2727</v>
+        <v>2831</v>
       </c>
     </row>
     <row r="218" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7735,7 +7735,7 @@
         <v>18</v>
       </c>
       <c r="H218" s="7">
-        <v>1743</v>
+        <v>2967</v>
       </c>
     </row>
     <row r="219" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7761,7 +7761,7 @@
         <v>18</v>
       </c>
       <c r="H219" s="7">
-        <v>1676</v>
+        <v>3199</v>
       </c>
     </row>
     <row r="220" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7787,7 +7787,7 @@
         <v>18</v>
       </c>
       <c r="H220" s="7">
-        <v>1891</v>
+        <v>3081</v>
       </c>
     </row>
     <row r="221" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7813,7 +7813,7 @@
         <v>18</v>
       </c>
       <c r="H221" s="7">
-        <v>2012</v>
+        <v>2938</v>
       </c>
     </row>
     <row r="222" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7839,7 +7839,7 @@
         <v>18</v>
       </c>
       <c r="H222" s="7">
-        <v>2460</v>
+        <v>3265</v>
       </c>
     </row>
     <row r="223" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7865,7 +7865,7 @@
         <v>18</v>
       </c>
       <c r="H223" s="7">
-        <v>1757</v>
+        <v>3375</v>
       </c>
     </row>
     <row r="224" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7891,7 +7891,7 @@
         <v>18</v>
       </c>
       <c r="H224" s="7">
-        <v>1767</v>
+        <v>2867</v>
       </c>
     </row>
     <row r="225" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7917,7 +7917,7 @@
         <v>18</v>
       </c>
       <c r="H225" s="7">
-        <v>1851</v>
+        <v>3286</v>
       </c>
     </row>
     <row r="226" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7943,7 +7943,7 @@
         <v>18</v>
       </c>
       <c r="H226" s="7">
-        <v>3287</v>
+        <v>3305</v>
       </c>
     </row>
     <row r="227" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7969,7 +7969,7 @@
         <v>18</v>
       </c>
       <c r="H227" s="7">
-        <v>3194</v>
+        <v>3294</v>
       </c>
     </row>
     <row r="228" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -7995,7 +7995,7 @@
         <v>18</v>
       </c>
       <c r="H228" s="7">
-        <v>2465</v>
+        <v>3349</v>
       </c>
     </row>
     <row r="229" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8021,7 +8021,7 @@
         <v>18</v>
       </c>
       <c r="H229" s="7">
-        <v>2783</v>
+        <v>3512</v>
       </c>
     </row>
     <row r="230" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8047,7 +8047,7 @@
         <v>18</v>
       </c>
       <c r="H230" s="7">
-        <v>3290</v>
+        <v>3603</v>
       </c>
     </row>
     <row r="231" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8073,7 +8073,7 @@
         <v>18</v>
       </c>
       <c r="H231" s="7">
-        <v>2732</v>
+        <v>3262</v>
       </c>
     </row>
     <row r="232" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8099,7 +8099,7 @@
         <v>18</v>
       </c>
       <c r="H232" s="7">
-        <v>1908</v>
+        <v>3045</v>
       </c>
     </row>
     <row r="233" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8125,7 +8125,7 @@
         <v>18</v>
       </c>
       <c r="H233" s="7">
-        <v>3329</v>
+        <v>2908</v>
       </c>
     </row>
     <row r="234" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8151,7 +8151,7 @@
         <v>18</v>
       </c>
       <c r="H234" s="7">
-        <v>3157</v>
+        <v>3230</v>
       </c>
     </row>
     <row r="235" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8177,7 +8177,7 @@
         <v>18</v>
       </c>
       <c r="H235" s="7">
-        <v>2806</v>
+        <v>2881</v>
       </c>
     </row>
     <row r="236" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8203,7 +8203,7 @@
         <v>18</v>
       </c>
       <c r="H236" s="7">
-        <v>1914</v>
+        <v>3534</v>
       </c>
     </row>
     <row r="237" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8229,7 +8229,7 @@
         <v>18</v>
       </c>
       <c r="H237" s="7">
-        <v>2587</v>
+        <v>3195</v>
       </c>
     </row>
     <row r="238" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8255,7 +8255,7 @@
         <v>18</v>
       </c>
       <c r="H238" s="7">
-        <v>2459</v>
+        <v>3624</v>
       </c>
     </row>
     <row r="239" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8281,7 +8281,7 @@
         <v>18</v>
       </c>
       <c r="H239" s="7">
-        <v>3055</v>
+        <v>4280</v>
       </c>
     </row>
     <row r="240" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8307,7 +8307,7 @@
         <v>18</v>
       </c>
       <c r="H240" s="7">
-        <v>1714</v>
+        <v>3976</v>
       </c>
     </row>
     <row r="241" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8333,7 +8333,7 @@
         <v>18</v>
       </c>
       <c r="H241" s="7">
-        <v>1805</v>
+        <v>3641</v>
       </c>
     </row>
     <row r="242" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8359,7 +8359,7 @@
         <v>18</v>
       </c>
       <c r="H242" s="7">
-        <v>1859</v>
+        <v>3453</v>
       </c>
     </row>
     <row r="243" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8385,7 +8385,7 @@
         <v>18</v>
       </c>
       <c r="H243" s="7">
-        <v>2094</v>
+        <v>3466</v>
       </c>
     </row>
     <row r="244" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8411,7 +8411,7 @@
         <v>18</v>
       </c>
       <c r="H244" s="7">
-        <v>1798</v>
+        <v>3790</v>
       </c>
     </row>
     <row r="245" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8437,7 +8437,7 @@
         <v>18</v>
       </c>
       <c r="H245" s="7">
-        <v>1799</v>
+        <v>3140</v>
       </c>
     </row>
     <row r="246" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8463,7 +8463,7 @@
         <v>18</v>
       </c>
       <c r="H246" s="7">
-        <v>1703</v>
+        <v>2984</v>
       </c>
     </row>
     <row r="247" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8489,7 +8489,7 @@
         <v>18</v>
       </c>
       <c r="H247" s="7">
-        <v>1689</v>
+        <v>3107</v>
       </c>
     </row>
     <row r="248" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8515,7 +8515,7 @@
         <v>18</v>
       </c>
       <c r="H248" s="7">
-        <v>1810</v>
+        <v>3230</v>
       </c>
     </row>
     <row r="249" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8541,7 +8541,7 @@
         <v>18</v>
       </c>
       <c r="H249" s="7">
-        <v>1808</v>
+        <v>2690</v>
       </c>
     </row>
     <row r="250" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8567,7 +8567,7 @@
         <v>18</v>
       </c>
       <c r="H250" s="7">
-        <v>1737</v>
+        <v>3855</v>
       </c>
     </row>
     <row r="251" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8593,7 +8593,7 @@
         <v>18</v>
       </c>
       <c r="H251" s="7">
-        <v>3111</v>
+        <v>2846</v>
       </c>
     </row>
     <row r="252" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8619,7 +8619,7 @@
         <v>18</v>
       </c>
       <c r="H252" s="7">
-        <v>3099</v>
+        <v>4802</v>
       </c>
     </row>
     <row r="253" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8645,7 +8645,7 @@
         <v>18</v>
       </c>
       <c r="H253" s="7">
-        <v>1902</v>
+        <v>3672</v>
       </c>
     </row>
     <row r="254" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8671,7 +8671,7 @@
         <v>18</v>
       </c>
       <c r="H254" s="7">
-        <v>1710</v>
+        <v>3375</v>
       </c>
     </row>
     <row r="255" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8697,7 +8697,7 @@
         <v>18</v>
       </c>
       <c r="H255" s="7">
-        <v>1775</v>
+        <v>3479</v>
       </c>
     </row>
     <row r="256" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8723,7 +8723,7 @@
         <v>18</v>
       </c>
       <c r="H256" s="7">
-        <v>1724</v>
+        <v>3909</v>
       </c>
     </row>
     <row r="257" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8749,7 +8749,7 @@
         <v>18</v>
       </c>
       <c r="H257" s="7">
-        <v>1719</v>
+        <v>3666</v>
       </c>
     </row>
     <row r="258" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8775,7 +8775,7 @@
         <v>18</v>
       </c>
       <c r="H258" s="7">
-        <v>1818</v>
+        <v>3642</v>
       </c>
     </row>
     <row r="259" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8801,7 +8801,7 @@
         <v>18</v>
       </c>
       <c r="H259" s="7">
-        <v>1801</v>
+        <v>3430</v>
       </c>
     </row>
     <row r="260" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8827,7 +8827,7 @@
         <v>18</v>
       </c>
       <c r="H260" s="7">
-        <v>1841</v>
+        <v>5873</v>
       </c>
     </row>
     <row r="261" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8853,7 +8853,7 @@
         <v>18</v>
       </c>
       <c r="H261" s="7">
-        <v>1756</v>
+        <v>4955</v>
       </c>
     </row>
     <row r="262" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8879,7 +8879,7 @@
         <v>18</v>
       </c>
       <c r="H262" s="7">
-        <v>1751</v>
+        <v>5094</v>
       </c>
     </row>
     <row r="263" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8905,7 +8905,7 @@
         <v>18</v>
       </c>
       <c r="H263" s="7">
-        <v>1795</v>
+        <v>5154</v>
       </c>
     </row>
     <row r="264" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8931,7 +8931,7 @@
         <v>18</v>
       </c>
       <c r="H264" s="7">
-        <v>1745</v>
+        <v>4013</v>
       </c>
     </row>
     <row r="265" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8957,7 +8957,7 @@
         <v>18</v>
       </c>
       <c r="H265" s="7">
-        <v>1889</v>
+        <v>4751</v>
       </c>
     </row>
     <row r="266" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -8983,7 +8983,7 @@
         <v>18</v>
       </c>
       <c r="H266" s="7">
-        <v>1775</v>
+        <v>4333</v>
       </c>
     </row>
     <row r="267" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9009,7 +9009,7 @@
         <v>18</v>
       </c>
       <c r="H267" s="7">
-        <v>1809</v>
+        <v>3807</v>
       </c>
     </row>
     <row r="268" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9035,7 +9035,7 @@
         <v>18</v>
       </c>
       <c r="H268" s="7">
-        <v>1834</v>
+        <v>4098</v>
       </c>
     </row>
     <row r="269" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9061,7 +9061,7 @@
         <v>18</v>
       </c>
       <c r="H269" s="7">
-        <v>1733</v>
+        <v>4541</v>
       </c>
     </row>
     <row r="270" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9087,7 +9087,7 @@
         <v>18</v>
       </c>
       <c r="H270" s="7">
-        <v>1800</v>
+        <v>3318</v>
       </c>
     </row>
     <row r="271" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9113,7 +9113,7 @@
         <v>18</v>
       </c>
       <c r="H271" s="7">
-        <v>2616</v>
+        <v>3748</v>
       </c>
     </row>
     <row r="272" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9139,7 +9139,7 @@
         <v>18</v>
       </c>
       <c r="H272" s="7">
-        <v>2646</v>
+        <v>3906</v>
       </c>
     </row>
     <row r="273" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9165,7 +9165,7 @@
         <v>18</v>
       </c>
       <c r="H273" s="7">
-        <v>1827</v>
+        <v>3628</v>
       </c>
     </row>
     <row r="274" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9191,7 +9191,7 @@
         <v>18</v>
       </c>
       <c r="H274" s="7">
-        <v>1872</v>
+        <v>5369</v>
       </c>
     </row>
     <row r="275" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9217,7 +9217,7 @@
         <v>18</v>
       </c>
       <c r="H275" s="7">
-        <v>1776</v>
+        <v>4374</v>
       </c>
     </row>
     <row r="276" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9243,7 +9243,7 @@
         <v>18</v>
       </c>
       <c r="H276" s="7">
-        <v>2318</v>
+        <v>3714</v>
       </c>
     </row>
     <row r="277" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9269,7 +9269,7 @@
         <v>18</v>
       </c>
       <c r="H277" s="7">
-        <v>3053</v>
+        <v>4508</v>
       </c>
     </row>
     <row r="278" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9295,7 +9295,7 @@
         <v>18</v>
       </c>
       <c r="H278" s="7">
-        <v>3144</v>
+        <v>4751</v>
       </c>
     </row>
     <row r="279" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9321,7 +9321,7 @@
         <v>18</v>
       </c>
       <c r="H279" s="7">
-        <v>2341</v>
+        <v>5283</v>
       </c>
     </row>
     <row r="280" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9347,7 +9347,7 @@
         <v>18</v>
       </c>
       <c r="H280" s="7">
-        <v>1856</v>
+        <v>3688</v>
       </c>
     </row>
     <row r="281" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9373,7 +9373,7 @@
         <v>18</v>
       </c>
       <c r="H281" s="7">
-        <v>1914</v>
+        <v>5713</v>
       </c>
     </row>
     <row r="282" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9399,7 +9399,7 @@
         <v>18</v>
       </c>
       <c r="H282" s="7">
-        <v>2498</v>
+        <v>4015</v>
       </c>
     </row>
     <row r="283" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9425,7 +9425,7 @@
         <v>18</v>
       </c>
       <c r="H283" s="7">
-        <v>2978</v>
+        <v>3474</v>
       </c>
     </row>
     <row r="284" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9451,7 +9451,7 @@
         <v>18</v>
       </c>
       <c r="H284" s="7">
-        <v>2360</v>
+        <v>3564</v>
       </c>
     </row>
     <row r="285" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9477,7 +9477,7 @@
         <v>18</v>
       </c>
       <c r="H285" s="7">
-        <v>1939</v>
+        <v>3620</v>
       </c>
     </row>
     <row r="286" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9503,7 +9503,7 @@
         <v>18</v>
       </c>
       <c r="H286" s="7">
-        <v>1804</v>
+        <v>3935</v>
       </c>
     </row>
     <row r="287" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9529,7 +9529,7 @@
         <v>18</v>
       </c>
       <c r="H287" s="7">
-        <v>1767</v>
+        <v>4276</v>
       </c>
     </row>
     <row r="288" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9555,7 +9555,7 @@
         <v>18</v>
       </c>
       <c r="H288" s="7">
-        <v>1889</v>
+        <v>3976</v>
       </c>
     </row>
     <row r="289" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9581,7 +9581,7 @@
         <v>18</v>
       </c>
       <c r="H289" s="7">
-        <v>1951</v>
+        <v>3806</v>
       </c>
     </row>
     <row r="290" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9607,7 +9607,7 @@
         <v>18</v>
       </c>
       <c r="H290" s="7">
-        <v>1764</v>
+        <v>3930</v>
       </c>
     </row>
     <row r="291" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9633,7 +9633,7 @@
         <v>18</v>
       </c>
       <c r="H291" s="7">
-        <v>2108</v>
+        <v>4048</v>
       </c>
     </row>
     <row r="292" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9659,7 +9659,7 @@
         <v>18</v>
       </c>
       <c r="H292" s="7">
-        <v>1883</v>
+        <v>3624</v>
       </c>
     </row>
     <row r="293" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9685,7 +9685,7 @@
         <v>18</v>
       </c>
       <c r="H293" s="7">
-        <v>1876</v>
+        <v>3697</v>
       </c>
     </row>
     <row r="294" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9711,7 +9711,7 @@
         <v>18</v>
       </c>
       <c r="H294" s="7">
-        <v>1761</v>
+        <v>3849</v>
       </c>
     </row>
     <row r="295" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9737,7 +9737,7 @@
         <v>18</v>
       </c>
       <c r="H295" s="7">
-        <v>1751</v>
+        <v>5038</v>
       </c>
     </row>
     <row r="296" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9763,7 +9763,7 @@
         <v>18</v>
       </c>
       <c r="H296" s="7">
-        <v>1878</v>
+        <v>3674</v>
       </c>
     </row>
     <row r="297" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9789,7 +9789,7 @@
         <v>18</v>
       </c>
       <c r="H297" s="7">
-        <v>2006</v>
+        <v>3363</v>
       </c>
     </row>
     <row r="298" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9815,7 +9815,7 @@
         <v>18</v>
       </c>
       <c r="H298" s="7">
-        <v>1773</v>
+        <v>4145</v>
       </c>
     </row>
     <row r="299" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9841,7 +9841,7 @@
         <v>18</v>
       </c>
       <c r="H299" s="7">
-        <v>1800</v>
+        <v>3462</v>
       </c>
     </row>
     <row r="300" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9867,7 +9867,7 @@
         <v>18</v>
       </c>
       <c r="H300" s="7">
-        <v>1838</v>
+        <v>2710</v>
       </c>
     </row>
     <row r="301" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9893,7 +9893,7 @@
         <v>18</v>
       </c>
       <c r="H301" s="7">
-        <v>1832</v>
+        <v>4962</v>
       </c>
     </row>
     <row r="302" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9919,7 +9919,7 @@
         <v>18</v>
       </c>
       <c r="H302" s="7">
-        <v>1828</v>
+        <v>3872</v>
       </c>
     </row>
     <row r="303" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9945,7 +9945,7 @@
         <v>18</v>
       </c>
       <c r="H303" s="7">
-        <v>1848</v>
+        <v>3417</v>
       </c>
     </row>
     <row r="304" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9971,7 +9971,7 @@
         <v>18</v>
       </c>
       <c r="H304" s="7">
-        <v>2055</v>
+        <v>3584</v>
       </c>
     </row>
     <row r="305" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -9997,7 +9997,7 @@
         <v>18</v>
       </c>
       <c r="H305" s="7">
-        <v>2854</v>
+        <v>3328</v>
       </c>
     </row>
     <row r="306" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -10023,7 +10023,7 @@
         <v>18</v>
       </c>
       <c r="H306" s="7">
-        <v>2682</v>
+        <v>3629</v>
       </c>
     </row>
   </sheetData>

</xml_diff>